<commit_message>
Hide Ultimate CEO section and rename Top CEO to TOP/ULTIMATE CEO EVENT SCORING
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/EventScoring.xlsx
+++ b/src/EventScoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mick/Documents/ApexGirl/CEO Calculators/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D23B0791-ABF7-2A4B-9B77-337B0DB9D754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A56DFE7-2BFA-3A41-B985-0E4CFE98B3C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="39480" yWindow="2640" windowWidth="32000" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,15 +62,9 @@
     <t>Vehicle</t>
   </si>
   <si>
-    <t>Use 1 item(s) to upgrade car parts</t>
-  </si>
-  <si>
     <t>Development</t>
   </si>
   <si>
-    <t>Use 1 item(s) to promote car</t>
-  </si>
-  <si>
     <t>Use Spark Plugs (Novice)</t>
   </si>
   <si>
@@ -258,6 +252,12 @@
   </si>
   <si>
     <t>Use Blueprint point</t>
+  </si>
+  <si>
+    <t>Upgrade Car Parts x1</t>
+  </si>
+  <si>
+    <t>Promote Car x1</t>
   </si>
 </sst>
 </file>
@@ -459,30 +459,30 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -834,26 +834,26 @@
   <sheetData>
     <row r="1" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="G1" s="27" t="s">
+      <c r="B1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="G1" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="M1" s="27" t="s">
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="M1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
     </row>
     <row r="2" spans="1:17" ht="6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="2"/>
@@ -868,47 +868,47 @@
       <c r="Q2" s="5"/>
     </row>
     <row r="3" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="26"/>
-      <c r="P3" s="26"/>
-      <c r="Q3" s="31"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="24"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="32"/>
     </row>
     <row r="4" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
+      <c r="B4" s="30" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
       <c r="E4" s="4"/>
       <c r="F4" s="3"/>
-      <c r="G4" s="28" t="s">
+      <c r="G4" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
       <c r="J4" s="2"/>
       <c r="K4" s="5"/>
       <c r="L4" s="3"/>
-      <c r="M4" s="28" t="s">
+      <c r="M4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="N4" s="26"/>
-      <c r="O4" s="26"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="5"/>
     </row>
@@ -957,7 +957,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>9</v>
+        <v>73</v>
       </c>
       <c r="C6" s="10">
         <v>500</v>
@@ -974,7 +974,7 @@
         <v>8</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>9</v>
+        <v>73</v>
       </c>
       <c r="I6" s="10">
         <v>500</v>
@@ -988,10 +988,10 @@
       </c>
       <c r="L6" s="10"/>
       <c r="M6" s="25" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N6" s="9" t="s">
-        <v>9</v>
+        <v>73</v>
       </c>
       <c r="O6" s="10">
         <v>500</v>
@@ -1005,9 +1005,9 @@
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A7" s="26"/>
+      <c r="A7" s="24"/>
       <c r="B7" s="9" t="s">
-        <v>11</v>
+        <v>74</v>
       </c>
       <c r="C7" s="10">
         <v>2500</v>
@@ -1020,9 +1020,9 @@
         <v>0</v>
       </c>
       <c r="F7" s="10"/>
-      <c r="G7" s="26"/>
+      <c r="G7" s="24"/>
       <c r="H7" s="9" t="s">
-        <v>11</v>
+        <v>74</v>
       </c>
       <c r="I7" s="10">
         <v>2500</v>
@@ -1035,9 +1035,9 @@
         <v>0</v>
       </c>
       <c r="L7" s="10"/>
-      <c r="M7" s="26"/>
+      <c r="M7" s="24"/>
       <c r="N7" s="9" t="s">
-        <v>11</v>
+        <v>74</v>
       </c>
       <c r="O7" s="10">
         <v>2500</v>
@@ -1051,9 +1051,9 @@
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A8" s="26"/>
+      <c r="A8" s="24"/>
       <c r="B8" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8" s="10">
         <v>1000</v>
@@ -1066,9 +1066,9 @@
         <v>0</v>
       </c>
       <c r="F8" s="10"/>
-      <c r="G8" s="26"/>
+      <c r="G8" s="24"/>
       <c r="H8" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I8" s="10">
         <v>1000</v>
@@ -1081,9 +1081,9 @@
         <v>0</v>
       </c>
       <c r="L8" s="10"/>
-      <c r="M8" s="26"/>
+      <c r="M8" s="24"/>
       <c r="N8" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O8" s="10">
         <v>400</v>
@@ -1097,9 +1097,9 @@
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="26"/>
+      <c r="A9" s="24"/>
       <c r="B9" s="9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C9" s="10">
         <v>10000</v>
@@ -1112,9 +1112,9 @@
         <v>0</v>
       </c>
       <c r="F9" s="10"/>
-      <c r="G9" s="26"/>
+      <c r="G9" s="24"/>
       <c r="H9" s="9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I9" s="10">
         <v>10000</v>
@@ -1127,9 +1127,9 @@
         <v>0</v>
       </c>
       <c r="L9" s="10"/>
-      <c r="M9" s="26"/>
+      <c r="M9" s="24"/>
       <c r="N9" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O9" s="10">
         <v>50000</v>
@@ -1143,9 +1143,9 @@
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A10" s="26"/>
+      <c r="A10" s="24"/>
       <c r="B10" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C10" s="10">
         <v>125000</v>
@@ -1158,9 +1158,9 @@
         <v>0</v>
       </c>
       <c r="F10" s="10"/>
-      <c r="G10" s="26"/>
+      <c r="G10" s="24"/>
       <c r="H10" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I10" s="10">
         <v>125000</v>
@@ -1173,9 +1173,9 @@
         <v>0</v>
       </c>
       <c r="L10" s="10"/>
-      <c r="M10" s="26"/>
+      <c r="M10" s="24"/>
       <c r="N10" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="O10" s="10">
         <v>125000</v>
@@ -1189,9 +1189,9 @@
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A11" s="26"/>
+      <c r="A11" s="24"/>
       <c r="B11" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C11" s="10">
         <v>1250000</v>
@@ -1204,9 +1204,9 @@
         <v>0</v>
       </c>
       <c r="F11" s="10"/>
-      <c r="G11" s="26"/>
+      <c r="G11" s="24"/>
       <c r="H11" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I11" s="10">
         <v>1250000</v>
@@ -1219,9 +1219,9 @@
         <v>0</v>
       </c>
       <c r="L11" s="10"/>
-      <c r="M11" s="26"/>
+      <c r="M11" s="24"/>
       <c r="N11" s="9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="O11" s="10">
         <v>4000</v>
@@ -1235,9 +1235,9 @@
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A12" s="26"/>
+      <c r="A12" s="24"/>
       <c r="B12" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C12" s="10">
         <v>15625000</v>
@@ -1250,9 +1250,9 @@
         <v>0</v>
       </c>
       <c r="F12" s="10"/>
-      <c r="G12" s="26"/>
+      <c r="G12" s="24"/>
       <c r="H12" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I12" s="10">
         <v>15625000</v>
@@ -1265,9 +1265,9 @@
         <v>0</v>
       </c>
       <c r="L12" s="10"/>
-      <c r="M12" s="26"/>
+      <c r="M12" s="24"/>
       <c r="N12" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O12" s="10">
         <v>500000</v>
@@ -1281,9 +1281,9 @@
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A13" s="26"/>
+      <c r="A13" s="24"/>
       <c r="B13" s="9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C13" s="10">
         <v>156250000</v>
@@ -1296,9 +1296,9 @@
         <v>0</v>
       </c>
       <c r="F13" s="10"/>
-      <c r="G13" s="26"/>
+      <c r="G13" s="24"/>
       <c r="H13" s="9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I13" s="10">
         <v>156250000</v>
@@ -1311,9 +1311,9 @@
         <v>0</v>
       </c>
       <c r="L13" s="10"/>
-      <c r="M13" s="26"/>
+      <c r="M13" s="24"/>
       <c r="N13" s="9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="O13" s="10">
         <v>62500000</v>
@@ -1327,9 +1327,9 @@
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A14" s="26"/>
+      <c r="A14" s="24"/>
       <c r="B14" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C14" s="10">
         <v>1</v>
@@ -1342,9 +1342,9 @@
         <v>0</v>
       </c>
       <c r="F14" s="10"/>
-      <c r="G14" s="26"/>
+      <c r="G14" s="24"/>
       <c r="H14" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I14" s="10">
         <v>1</v>
@@ -1357,9 +1357,9 @@
         <v>0</v>
       </c>
       <c r="L14" s="10"/>
-      <c r="M14" s="26"/>
+      <c r="M14" s="24"/>
       <c r="N14" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O14" s="10">
         <v>500</v>
@@ -1373,9 +1373,9 @@
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A15" s="26"/>
+      <c r="A15" s="24"/>
       <c r="B15" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C15" s="10">
         <v>50000</v>
@@ -1388,9 +1388,9 @@
         <v>0</v>
       </c>
       <c r="F15" s="10"/>
-      <c r="G15" s="26"/>
+      <c r="G15" s="24"/>
       <c r="H15" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I15" s="10">
         <v>50000</v>
@@ -1403,9 +1403,9 @@
         <v>0</v>
       </c>
       <c r="L15" s="10"/>
-      <c r="M15" s="26"/>
+      <c r="M15" s="24"/>
       <c r="N15" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="O15" s="10">
         <v>400</v>
@@ -1419,9 +1419,9 @@
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A16" s="26"/>
+      <c r="A16" s="24"/>
       <c r="B16" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C16" s="10">
         <v>1</v>
@@ -1434,9 +1434,9 @@
         <v>0</v>
       </c>
       <c r="F16" s="10"/>
-      <c r="G16" s="26"/>
+      <c r="G16" s="24"/>
       <c r="H16" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I16" s="10">
         <v>1</v>
@@ -1449,9 +1449,9 @@
         <v>0</v>
       </c>
       <c r="L16" s="10"/>
-      <c r="M16" s="26"/>
+      <c r="M16" s="24"/>
       <c r="N16" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="O16" s="10">
         <v>50000</v>
@@ -1465,9 +1465,9 @@
       </c>
     </row>
     <row r="17" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="26"/>
+      <c r="A17" s="24"/>
       <c r="B17" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C17" s="10">
         <v>10000</v>
@@ -1480,9 +1480,9 @@
         <v>0</v>
       </c>
       <c r="F17" s="10"/>
-      <c r="G17" s="26"/>
+      <c r="G17" s="24"/>
       <c r="H17" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I17" s="10">
         <v>10000</v>
@@ -1495,9 +1495,9 @@
         <v>0</v>
       </c>
       <c r="L17" s="10"/>
-      <c r="M17" s="26"/>
+      <c r="M17" s="24"/>
       <c r="N17" s="9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O17" s="10">
         <v>6250000</v>
@@ -1511,9 +1511,9 @@
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A18" s="26"/>
+      <c r="A18" s="24"/>
       <c r="B18" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C18" s="10">
         <v>40000</v>
@@ -1526,9 +1526,9 @@
         <v>0</v>
       </c>
       <c r="F18" s="10"/>
-      <c r="G18" s="26"/>
+      <c r="G18" s="24"/>
       <c r="H18" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I18" s="10">
         <v>40000</v>
@@ -1541,9 +1541,9 @@
         <v>0</v>
       </c>
       <c r="L18" s="10"/>
-      <c r="M18" s="26"/>
+      <c r="M18" s="24"/>
       <c r="N18" s="9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="O18" s="10">
         <v>4000</v>
@@ -1558,10 +1558,10 @@
     </row>
     <row r="19" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="12"/>
-      <c r="B19" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" s="24"/>
+      <c r="B19" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="27"/>
       <c r="D19" s="13"/>
       <c r="E19" s="14">
         <f>SUM(E6:E18)</f>
@@ -1569,19 +1569,19 @@
       </c>
       <c r="F19" s="15"/>
       <c r="G19" s="12"/>
-      <c r="H19" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="I19" s="24"/>
+      <c r="H19" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="I19" s="27"/>
       <c r="J19" s="13"/>
       <c r="K19" s="14">
         <f>SUM(K6:K18)</f>
         <v>0</v>
       </c>
       <c r="L19" s="15"/>
-      <c r="M19" s="26"/>
+      <c r="M19" s="24"/>
       <c r="N19" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="O19" s="10">
         <v>500000</v>
@@ -1596,10 +1596,10 @@
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C20" s="10">
         <v>500</v>
@@ -1613,10 +1613,10 @@
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="25" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I20" s="10">
         <v>500</v>
@@ -1629,9 +1629,9 @@
         <v>0</v>
       </c>
       <c r="L20" s="5"/>
-      <c r="M20" s="26"/>
+      <c r="M20" s="24"/>
       <c r="N20" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="O20" s="10">
         <v>62500000</v>
@@ -1645,9 +1645,9 @@
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A21" s="26"/>
+      <c r="A21" s="24"/>
       <c r="B21" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C21" s="10">
         <v>1000</v>
@@ -1660,9 +1660,9 @@
         <v>0</v>
       </c>
       <c r="F21" s="5"/>
-      <c r="G21" s="26"/>
+      <c r="G21" s="24"/>
       <c r="H21" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I21" s="10">
         <v>1000</v>
@@ -1675,9 +1675,9 @@
         <v>0</v>
       </c>
       <c r="L21" s="5"/>
-      <c r="M21" s="26"/>
+      <c r="M21" s="24"/>
       <c r="N21" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="O21" s="10">
         <v>1</v>
@@ -1691,9 +1691,9 @@
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A22" s="26"/>
+      <c r="A22" s="24"/>
       <c r="B22" s="9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C22" s="10">
         <v>10000</v>
@@ -1706,9 +1706,9 @@
         <v>0</v>
       </c>
       <c r="F22" s="5"/>
-      <c r="G22" s="26"/>
+      <c r="G22" s="24"/>
       <c r="H22" s="9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I22" s="10">
         <v>10000</v>
@@ -1721,9 +1721,9 @@
         <v>0</v>
       </c>
       <c r="L22" s="5"/>
-      <c r="M22" s="26"/>
+      <c r="M22" s="24"/>
       <c r="N22" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O22" s="10">
         <v>50000</v>
@@ -1737,9 +1737,9 @@
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A23" s="26"/>
+      <c r="A23" s="24"/>
       <c r="B23" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C23" s="10">
         <v>125000</v>
@@ -1752,9 +1752,9 @@
         <v>0</v>
       </c>
       <c r="F23" s="5"/>
-      <c r="G23" s="26"/>
+      <c r="G23" s="24"/>
       <c r="H23" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I23" s="10">
         <v>125000</v>
@@ -1767,9 +1767,9 @@
         <v>0</v>
       </c>
       <c r="L23" s="5"/>
-      <c r="M23" s="26"/>
+      <c r="M23" s="24"/>
       <c r="N23" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="O23" s="10">
         <v>1</v>
@@ -1783,9 +1783,9 @@
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A24" s="26"/>
+      <c r="A24" s="24"/>
       <c r="B24" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C24" s="10">
         <v>1250000</v>
@@ -1798,9 +1798,9 @@
         <v>0</v>
       </c>
       <c r="F24" s="5"/>
-      <c r="G24" s="26"/>
+      <c r="G24" s="24"/>
       <c r="H24" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I24" s="10">
         <v>1250000</v>
@@ -1813,9 +1813,9 @@
         <v>0</v>
       </c>
       <c r="L24" s="5"/>
-      <c r="M24" s="26"/>
+      <c r="M24" s="24"/>
       <c r="N24" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="O24" s="10">
         <v>10000</v>
@@ -1829,9 +1829,9 @@
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A25" s="26"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C25" s="10">
         <v>15625000</v>
@@ -1844,9 +1844,9 @@
         <v>0</v>
       </c>
       <c r="F25" s="5"/>
-      <c r="G25" s="26"/>
+      <c r="G25" s="24"/>
       <c r="H25" s="9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I25" s="10">
         <v>15625000</v>
@@ -1859,9 +1859,9 @@
         <v>0</v>
       </c>
       <c r="L25" s="5"/>
-      <c r="M25" s="26"/>
+      <c r="M25" s="24"/>
       <c r="N25" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="O25" s="10">
         <v>40000</v>
@@ -1875,9 +1875,9 @@
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A26" s="26"/>
+      <c r="A26" s="24"/>
       <c r="B26" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C26" s="10">
         <v>156250000</v>
@@ -1890,9 +1890,9 @@
         <v>0</v>
       </c>
       <c r="F26" s="5"/>
-      <c r="G26" s="26"/>
+      <c r="G26" s="24"/>
       <c r="H26" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I26" s="10">
         <v>156250000</v>
@@ -1905,9 +1905,9 @@
         <v>0</v>
       </c>
       <c r="L26" s="5"/>
-      <c r="M26" s="26"/>
+      <c r="M26" s="24"/>
       <c r="N26" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="O26" s="10">
         <v>8</v>
@@ -1921,9 +1921,9 @@
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A27" s="26"/>
+      <c r="A27" s="24"/>
       <c r="B27" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C27" s="10">
         <v>1</v>
@@ -1936,9 +1936,9 @@
         <v>0</v>
       </c>
       <c r="F27" s="5"/>
-      <c r="G27" s="26"/>
+      <c r="G27" s="24"/>
       <c r="H27" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I27" s="10">
         <v>1</v>
@@ -1951,10 +1951,10 @@
         <v>0</v>
       </c>
       <c r="L27" s="5"/>
-      <c r="N27" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="O27" s="24"/>
+      <c r="N27" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="O27" s="27"/>
       <c r="P27" s="13"/>
       <c r="Q27" s="14">
         <f>SUM(Q6:Q26)</f>
@@ -1962,9 +1962,9 @@
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A28" s="26"/>
+      <c r="A28" s="24"/>
       <c r="B28" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C28" s="10">
         <v>50000</v>
@@ -1977,9 +1977,9 @@
         <v>0</v>
       </c>
       <c r="F28" s="5"/>
-      <c r="G28" s="26"/>
+      <c r="G28" s="24"/>
       <c r="H28" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I28" s="10">
         <v>50000</v>
@@ -1993,10 +1993,10 @@
       </c>
       <c r="L28" s="5"/>
       <c r="M28" s="25" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="N28" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="O28" s="20">
         <v>500</v>
@@ -2010,9 +2010,9 @@
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A29" s="26"/>
+      <c r="A29" s="24"/>
       <c r="B29" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C29" s="10">
         <v>1</v>
@@ -2025,9 +2025,9 @@
         <v>0</v>
       </c>
       <c r="F29" s="5"/>
-      <c r="G29" s="26"/>
+      <c r="G29" s="24"/>
       <c r="H29" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I29" s="10">
         <v>1</v>
@@ -2040,9 +2040,9 @@
         <v>0</v>
       </c>
       <c r="L29" s="5"/>
-      <c r="M29" s="26"/>
+      <c r="M29" s="24"/>
       <c r="N29" s="9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O29" s="20">
         <v>1000</v>
@@ -2056,9 +2056,9 @@
       </c>
     </row>
     <row r="30" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="26"/>
+      <c r="A30" s="24"/>
       <c r="B30" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C30" s="10">
         <v>10000</v>
@@ -2071,9 +2071,9 @@
         <v>0</v>
       </c>
       <c r="F30" s="5"/>
-      <c r="G30" s="26"/>
+      <c r="G30" s="24"/>
       <c r="H30" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I30" s="10">
         <v>10000</v>
@@ -2086,9 +2086,9 @@
         <v>0</v>
       </c>
       <c r="L30" s="5"/>
-      <c r="M30" s="26"/>
+      <c r="M30" s="24"/>
       <c r="N30" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="O30" s="9">
         <v>1000</v>
@@ -2102,9 +2102,9 @@
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A31" s="26"/>
+      <c r="A31" s="24"/>
       <c r="B31" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C31" s="10">
         <v>40000</v>
@@ -2117,9 +2117,9 @@
         <v>0</v>
       </c>
       <c r="F31" s="5"/>
-      <c r="G31" s="26"/>
+      <c r="G31" s="24"/>
       <c r="H31" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I31" s="10">
         <v>40000</v>
@@ -2132,9 +2132,9 @@
         <v>0</v>
       </c>
       <c r="L31" s="5"/>
-      <c r="M31" s="26"/>
+      <c r="M31" s="24"/>
       <c r="N31" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="O31" s="9">
         <v>125000</v>
@@ -2149,10 +2149,10 @@
     </row>
     <row r="32" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="17"/>
-      <c r="B32" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C32" s="24"/>
+      <c r="B32" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="27"/>
       <c r="D32" s="13"/>
       <c r="E32" s="18">
         <f>SUM(E20:E31)</f>
@@ -2160,19 +2160,19 @@
       </c>
       <c r="F32" s="19"/>
       <c r="G32" s="17"/>
-      <c r="H32" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="I32" s="24"/>
+      <c r="H32" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="I32" s="27"/>
       <c r="J32" s="13"/>
       <c r="K32" s="18">
         <f>SUM(K20:K31)</f>
         <v>0</v>
       </c>
       <c r="L32" s="19"/>
-      <c r="M32" s="26"/>
+      <c r="M32" s="24"/>
       <c r="N32" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="O32" s="9">
         <v>15625000</v>
@@ -2187,10 +2187,10 @@
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" s="25" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C33" s="20">
         <v>500</v>
@@ -2204,10 +2204,10 @@
       </c>
       <c r="F33" s="5"/>
       <c r="G33" s="25" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I33" s="20">
         <v>500</v>
@@ -2220,9 +2220,9 @@
         <v>0</v>
       </c>
       <c r="L33" s="5"/>
-      <c r="M33" s="26"/>
+      <c r="M33" s="24"/>
       <c r="N33" s="9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="O33" s="9">
         <v>10000</v>
@@ -2236,9 +2236,9 @@
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A34" s="26"/>
+      <c r="A34" s="24"/>
       <c r="B34" s="9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C34" s="20">
         <v>1000</v>
@@ -2251,9 +2251,9 @@
         <v>0</v>
       </c>
       <c r="F34" s="5"/>
-      <c r="G34" s="26"/>
+      <c r="G34" s="24"/>
       <c r="H34" s="9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I34" s="20">
         <v>1000</v>
@@ -2266,9 +2266,9 @@
         <v>0</v>
       </c>
       <c r="L34" s="5"/>
-      <c r="M34" s="26"/>
+      <c r="M34" s="24"/>
       <c r="N34" s="9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="O34" s="9">
         <v>1250000</v>
@@ -2282,9 +2282,9 @@
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A35" s="26"/>
+      <c r="A35" s="24"/>
       <c r="B35" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C35" s="9">
         <v>2000</v>
@@ -2297,9 +2297,9 @@
         <v>0</v>
       </c>
       <c r="F35" s="5"/>
-      <c r="G35" s="26"/>
+      <c r="G35" s="24"/>
       <c r="H35" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I35" s="9">
         <v>2000</v>
@@ -2312,9 +2312,9 @@
         <v>0</v>
       </c>
       <c r="L35" s="5"/>
-      <c r="M35" s="26"/>
+      <c r="M35" s="24"/>
       <c r="N35" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O35" s="9">
         <v>156250000</v>
@@ -2328,9 +2328,9 @@
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A36" s="26"/>
+      <c r="A36" s="24"/>
       <c r="B36" s="9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C36">
         <v>20000</v>
@@ -2343,9 +2343,9 @@
         <v>0</v>
       </c>
       <c r="F36" s="5"/>
-      <c r="G36" s="26"/>
+      <c r="G36" s="24"/>
       <c r="H36" s="9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I36">
         <v>20000</v>
@@ -2358,9 +2358,9 @@
         <v>0</v>
       </c>
       <c r="L36" s="5"/>
-      <c r="M36" s="26"/>
+      <c r="M36" s="24"/>
       <c r="N36" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O36" s="9">
         <v>500</v>
@@ -2374,9 +2374,9 @@
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A37" s="26"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C37">
         <v>250000</v>
@@ -2389,9 +2389,9 @@
         <v>0</v>
       </c>
       <c r="F37" s="5"/>
-      <c r="G37" s="26"/>
+      <c r="G37" s="24"/>
       <c r="H37" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I37">
         <v>250000</v>
@@ -2404,9 +2404,9 @@
         <v>0</v>
       </c>
       <c r="L37" s="5"/>
-      <c r="M37" s="26"/>
+      <c r="M37" s="24"/>
       <c r="N37" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="O37" s="9">
         <v>5000</v>
@@ -2420,9 +2420,9 @@
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A38" s="26"/>
+      <c r="A38" s="24"/>
       <c r="B38" s="9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C38">
         <v>2500000</v>
@@ -2435,9 +2435,9 @@
         <v>0</v>
       </c>
       <c r="F38" s="5"/>
-      <c r="G38" s="26"/>
+      <c r="G38" s="24"/>
       <c r="H38" s="9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I38">
         <v>2500000</v>
@@ -2450,9 +2450,9 @@
         <v>0</v>
       </c>
       <c r="L38" s="5"/>
-      <c r="M38" s="26"/>
+      <c r="M38" s="24"/>
       <c r="N38" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="O38" s="9">
         <v>1000</v>
@@ -2466,9 +2466,9 @@
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A39" s="26"/>
+      <c r="A39" s="24"/>
       <c r="B39" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C39">
         <v>31250000</v>
@@ -2481,9 +2481,9 @@
         <v>0</v>
       </c>
       <c r="F39" s="5"/>
-      <c r="G39" s="26"/>
+      <c r="G39" s="24"/>
       <c r="H39" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I39">
         <v>31250000</v>
@@ -2496,9 +2496,9 @@
         <v>0</v>
       </c>
       <c r="L39" s="5"/>
-      <c r="M39" s="26"/>
+      <c r="M39" s="24"/>
       <c r="N39" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O39" s="9">
         <v>125000</v>
@@ -2512,9 +2512,9 @@
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A40" s="26"/>
+      <c r="A40" s="24"/>
       <c r="B40" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C40">
         <v>312500000</v>
@@ -2527,9 +2527,9 @@
         <v>0</v>
       </c>
       <c r="F40" s="5"/>
-      <c r="G40" s="26"/>
+      <c r="G40" s="24"/>
       <c r="H40" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I40">
         <v>312500000</v>
@@ -2542,9 +2542,9 @@
         <v>0</v>
       </c>
       <c r="L40" s="5"/>
-      <c r="M40" s="26"/>
+      <c r="M40" s="24"/>
       <c r="N40" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="O40">
         <v>15625000</v>
@@ -2558,9 +2558,9 @@
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A41" s="26"/>
+      <c r="A41" s="24"/>
       <c r="B41" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -2573,9 +2573,9 @@
         <v>0</v>
       </c>
       <c r="F41" s="5"/>
-      <c r="G41" s="26"/>
+      <c r="G41" s="24"/>
       <c r="H41" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I41">
         <v>1</v>
@@ -2588,9 +2588,9 @@
         <v>0</v>
       </c>
       <c r="L41" s="5"/>
-      <c r="M41" s="26"/>
+      <c r="M41" s="24"/>
       <c r="N41" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="O41">
         <v>10000</v>
@@ -2604,9 +2604,9 @@
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A42" s="26"/>
+      <c r="A42" s="24"/>
       <c r="B42" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C42">
         <v>50000</v>
@@ -2619,9 +2619,9 @@
         <v>0</v>
       </c>
       <c r="F42" s="5"/>
-      <c r="G42" s="26"/>
+      <c r="G42" s="24"/>
       <c r="H42" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I42">
         <v>50000</v>
@@ -2634,9 +2634,9 @@
         <v>0</v>
       </c>
       <c r="L42" s="5"/>
-      <c r="M42" s="26"/>
+      <c r="M42" s="24"/>
       <c r="N42" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="O42">
         <v>1250000</v>
@@ -2650,9 +2650,9 @@
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A43" s="26"/>
+      <c r="A43" s="24"/>
       <c r="B43" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -2665,9 +2665,9 @@
         <v>0</v>
       </c>
       <c r="F43" s="5"/>
-      <c r="G43" s="26"/>
+      <c r="G43" s="24"/>
       <c r="H43" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I43">
         <v>1</v>
@@ -2680,9 +2680,9 @@
         <v>0</v>
       </c>
       <c r="L43" s="5"/>
-      <c r="M43" s="26"/>
+      <c r="M43" s="24"/>
       <c r="N43" s="9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O43">
         <v>156250000</v>
@@ -2696,9 +2696,9 @@
       </c>
     </row>
     <row r="44" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="26"/>
+      <c r="A44" s="24"/>
       <c r="B44" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C44">
         <v>10000</v>
@@ -2711,9 +2711,9 @@
         <v>0</v>
       </c>
       <c r="F44" s="5"/>
-      <c r="G44" s="26"/>
+      <c r="G44" s="24"/>
       <c r="H44" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I44">
         <v>10000</v>
@@ -2726,9 +2726,9 @@
         <v>0</v>
       </c>
       <c r="L44" s="5"/>
-      <c r="M44" s="26"/>
+      <c r="M44" s="24"/>
       <c r="N44" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="O44">
         <v>1</v>
@@ -2742,9 +2742,9 @@
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A45" s="26"/>
+      <c r="A45" s="24"/>
       <c r="B45" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C45">
         <v>40000</v>
@@ -2757,9 +2757,9 @@
         <v>0</v>
       </c>
       <c r="F45" s="5"/>
-      <c r="G45" s="26"/>
+      <c r="G45" s="24"/>
       <c r="H45" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I45">
         <v>40000</v>
@@ -2772,9 +2772,9 @@
         <v>0</v>
       </c>
       <c r="L45" s="5"/>
-      <c r="M45" s="26"/>
+      <c r="M45" s="24"/>
       <c r="N45" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O45">
         <v>50000</v>
@@ -2789,10 +2789,10 @@
     </row>
     <row r="46" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
-      <c r="B46" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="C46" s="24"/>
+      <c r="B46" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" s="27"/>
       <c r="D46" s="13"/>
       <c r="E46" s="18">
         <f>SUM(E33:E45)</f>
@@ -2800,19 +2800,19 @@
       </c>
       <c r="F46" s="19"/>
       <c r="G46" s="13"/>
-      <c r="H46" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="I46" s="24"/>
+      <c r="H46" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="I46" s="27"/>
       <c r="J46" s="13"/>
       <c r="K46" s="18">
         <f>SUM(K33:K45)</f>
         <v>0</v>
       </c>
       <c r="L46" s="19"/>
-      <c r="M46" s="26"/>
+      <c r="M46" s="24"/>
       <c r="N46" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="O46">
         <v>1</v>
@@ -2826,11 +2826,11 @@
       </c>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A47" s="32" t="s">
-        <v>52</v>
+      <c r="A47" s="29" t="s">
+        <v>50</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C47">
         <v>37500</v>
@@ -2843,11 +2843,11 @@
         <v>0</v>
       </c>
       <c r="F47" s="5"/>
-      <c r="G47" s="32" t="s">
-        <v>52</v>
+      <c r="G47" s="29" t="s">
+        <v>50</v>
       </c>
       <c r="H47" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I47">
         <v>37500</v>
@@ -2860,9 +2860,9 @@
         <v>0</v>
       </c>
       <c r="L47" s="5"/>
-      <c r="M47" s="26"/>
+      <c r="M47" s="24"/>
       <c r="N47" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="O47">
         <v>10000</v>
@@ -2876,9 +2876,9 @@
       </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A48" s="26"/>
+      <c r="A48" s="24"/>
       <c r="B48" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C48">
         <v>500</v>
@@ -2891,9 +2891,9 @@
         <v>0</v>
       </c>
       <c r="F48" s="5"/>
-      <c r="G48" s="26"/>
+      <c r="G48" s="24"/>
       <c r="H48" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I48">
         <v>500</v>
@@ -2906,9 +2906,9 @@
         <v>0</v>
       </c>
       <c r="L48" s="5"/>
-      <c r="M48" s="26"/>
+      <c r="M48" s="24"/>
       <c r="N48" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="O48">
         <v>40000</v>
@@ -2922,9 +2922,9 @@
       </c>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A49" s="26"/>
+      <c r="A49" s="24"/>
       <c r="B49" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C49">
         <v>5000</v>
@@ -2937,9 +2937,9 @@
         <v>0</v>
       </c>
       <c r="F49" s="5"/>
-      <c r="G49" s="26"/>
+      <c r="G49" s="24"/>
       <c r="H49" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I49">
         <v>5000</v>
@@ -2954,7 +2954,7 @@
       <c r="L49" s="5"/>
       <c r="M49" s="8"/>
       <c r="N49" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="O49">
         <v>8</v>
@@ -2968,9 +2968,9 @@
       </c>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A50" s="26"/>
+      <c r="A50" s="24"/>
       <c r="B50" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C50">
         <v>2000</v>
@@ -2983,9 +2983,9 @@
         <v>0</v>
       </c>
       <c r="F50" s="5"/>
-      <c r="G50" s="26"/>
+      <c r="G50" s="24"/>
       <c r="H50" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I50">
         <v>2000</v>
@@ -2998,10 +2998,10 @@
         <v>0</v>
       </c>
       <c r="L50" s="5"/>
-      <c r="N50" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="O50" s="24"/>
+      <c r="N50" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="O50" s="27"/>
       <c r="P50" s="13"/>
       <c r="Q50" s="18">
         <f>SUM(Q28:Q49)</f>
@@ -3009,9 +3009,9 @@
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A51" s="26"/>
+      <c r="A51" s="24"/>
       <c r="B51" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C51">
         <v>20000</v>
@@ -3024,9 +3024,9 @@
         <v>0</v>
       </c>
       <c r="F51" s="5"/>
-      <c r="G51" s="26"/>
+      <c r="G51" s="24"/>
       <c r="H51" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I51">
         <v>20000</v>
@@ -3040,10 +3040,10 @@
       </c>
       <c r="L51" s="5"/>
       <c r="M51" s="25" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="O51" s="20">
         <v>60000</v>
@@ -3057,9 +3057,9 @@
       </c>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A52" s="26"/>
+      <c r="A52" s="24"/>
       <c r="B52" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C52">
         <v>250000</v>
@@ -3072,9 +3072,9 @@
         <v>0</v>
       </c>
       <c r="F52" s="5"/>
-      <c r="G52" s="26"/>
+      <c r="G52" s="24"/>
       <c r="H52" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I52">
         <v>250000</v>
@@ -3087,9 +3087,9 @@
         <v>0</v>
       </c>
       <c r="L52" s="5"/>
-      <c r="M52" s="26"/>
+      <c r="M52" s="24"/>
       <c r="N52" s="9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="O52" s="20">
         <v>60000</v>
@@ -3103,9 +3103,9 @@
       </c>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A53" s="26"/>
+      <c r="A53" s="24"/>
       <c r="B53" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C53">
         <v>2500000</v>
@@ -3118,9 +3118,9 @@
         <v>0</v>
       </c>
       <c r="F53" s="5"/>
-      <c r="G53" s="26"/>
+      <c r="G53" s="24"/>
       <c r="H53" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I53">
         <v>2500000</v>
@@ -3133,9 +3133,9 @@
         <v>0</v>
       </c>
       <c r="L53" s="5"/>
-      <c r="M53" s="26"/>
+      <c r="M53" s="24"/>
       <c r="N53" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O53" s="9">
         <v>5</v>
@@ -3149,9 +3149,9 @@
       </c>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A54" s="26"/>
+      <c r="A54" s="24"/>
       <c r="B54" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C54">
         <v>31250000</v>
@@ -3164,9 +3164,9 @@
         <v>0</v>
       </c>
       <c r="F54" s="5"/>
-      <c r="G54" s="26"/>
+      <c r="G54" s="24"/>
       <c r="H54" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I54">
         <v>31250000</v>
@@ -3179,9 +3179,9 @@
         <v>0</v>
       </c>
       <c r="L54" s="5"/>
-      <c r="M54" s="26"/>
+      <c r="M54" s="24"/>
       <c r="N54" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="O54" s="9">
         <v>1500</v>
@@ -3195,9 +3195,9 @@
       </c>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A55" s="26"/>
+      <c r="A55" s="24"/>
       <c r="B55" s="9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C55">
         <v>312500000</v>
@@ -3210,9 +3210,9 @@
         <v>0</v>
       </c>
       <c r="F55" s="5"/>
-      <c r="G55" s="26"/>
+      <c r="G55" s="24"/>
       <c r="H55" s="9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I55">
         <v>312500000</v>
@@ -3225,9 +3225,9 @@
         <v>0</v>
       </c>
       <c r="L55" s="5"/>
-      <c r="M55" s="26"/>
+      <c r="M55" s="24"/>
       <c r="N55" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O55" s="9">
         <v>4000</v>
@@ -3241,9 +3241,9 @@
       </c>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A56" s="26"/>
+      <c r="A56" s="24"/>
       <c r="B56" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -3256,9 +3256,9 @@
         <v>0</v>
       </c>
       <c r="F56" s="5"/>
-      <c r="G56" s="26"/>
+      <c r="G56" s="24"/>
       <c r="H56" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I56">
         <v>1</v>
@@ -3271,9 +3271,9 @@
         <v>0</v>
       </c>
       <c r="L56" s="5"/>
-      <c r="M56" s="26"/>
+      <c r="M56" s="24"/>
       <c r="N56" s="9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="O56" s="9">
         <v>4000</v>
@@ -3287,9 +3287,9 @@
       </c>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A57" s="26"/>
+      <c r="A57" s="24"/>
       <c r="B57" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C57">
         <v>50000</v>
@@ -3302,9 +3302,9 @@
         <v>0</v>
       </c>
       <c r="F57" s="5"/>
-      <c r="G57" s="26"/>
+      <c r="G57" s="24"/>
       <c r="H57" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I57">
         <v>50000</v>
@@ -3317,9 +3317,9 @@
         <v>0</v>
       </c>
       <c r="L57" s="5"/>
-      <c r="M57" s="26"/>
+      <c r="M57" s="24"/>
       <c r="N57" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="O57" s="9">
         <v>25000</v>
@@ -3333,9 +3333,9 @@
       </c>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A58" s="26"/>
+      <c r="A58" s="24"/>
       <c r="B58" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -3348,9 +3348,9 @@
         <v>0</v>
       </c>
       <c r="F58" s="5"/>
-      <c r="G58" s="26"/>
+      <c r="G58" s="24"/>
       <c r="H58" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I58">
         <v>1</v>
@@ -3363,9 +3363,9 @@
         <v>0</v>
       </c>
       <c r="L58" s="5"/>
-      <c r="M58" s="26"/>
+      <c r="M58" s="24"/>
       <c r="N58" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="O58">
         <v>1</v>
@@ -3379,9 +3379,9 @@
       </c>
     </row>
     <row r="59" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="24"/>
+      <c r="A59" s="27"/>
       <c r="B59" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C59">
         <v>10000</v>
@@ -3394,9 +3394,9 @@
         <v>0</v>
       </c>
       <c r="F59" s="5"/>
-      <c r="G59" s="24"/>
+      <c r="G59" s="27"/>
       <c r="H59" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I59">
         <v>10000</v>
@@ -3409,9 +3409,9 @@
         <v>0</v>
       </c>
       <c r="L59" s="5"/>
-      <c r="M59" s="26"/>
+      <c r="M59" s="24"/>
       <c r="N59" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O59">
         <v>50000</v>
@@ -3427,7 +3427,7 @@
     <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60" s="8"/>
       <c r="B60" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C60">
         <v>40000</v>
@@ -3442,7 +3442,7 @@
       <c r="F60" s="5"/>
       <c r="G60" s="8"/>
       <c r="H60" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I60">
         <v>40000</v>
@@ -3455,9 +3455,9 @@
         <v>0</v>
       </c>
       <c r="L60" s="5"/>
-      <c r="M60" s="26"/>
+      <c r="M60" s="24"/>
       <c r="N60" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="O60">
         <v>1</v>
@@ -3472,10 +3472,10 @@
     </row>
     <row r="61" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="13"/>
-      <c r="B61" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="C61" s="24"/>
+      <c r="B61" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C61" s="27"/>
       <c r="D61" s="13"/>
       <c r="E61" s="18">
         <f>SUM(E47:E60)</f>
@@ -3483,19 +3483,19 @@
       </c>
       <c r="F61" s="19"/>
       <c r="G61" s="13"/>
-      <c r="H61" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="I61" s="24"/>
+      <c r="H61" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="I61" s="27"/>
       <c r="J61" s="13"/>
       <c r="K61" s="18">
         <f>SUM(K47:K60)</f>
         <v>0</v>
       </c>
       <c r="L61" s="19"/>
-      <c r="M61" s="26"/>
+      <c r="M61" s="24"/>
       <c r="N61" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="O61">
         <v>10000</v>
@@ -3510,10 +3510,10 @@
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A62" s="25" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C62">
         <v>37500</v>
@@ -3527,10 +3527,10 @@
       </c>
       <c r="F62" s="5"/>
       <c r="G62" s="25" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I62">
         <v>37500</v>
@@ -3543,9 +3543,9 @@
         <v>0</v>
       </c>
       <c r="L62" s="5"/>
-      <c r="M62" s="26"/>
+      <c r="M62" s="24"/>
       <c r="N62" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="O62">
         <v>40000</v>
@@ -3559,9 +3559,9 @@
       </c>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A63" s="26"/>
+      <c r="A63" s="24"/>
       <c r="B63" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C63">
         <v>5</v>
@@ -3574,9 +3574,9 @@
         <v>0</v>
       </c>
       <c r="F63" s="5"/>
-      <c r="G63" s="26"/>
+      <c r="G63" s="24"/>
       <c r="H63" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I63">
         <v>5</v>
@@ -3589,9 +3589,9 @@
         <v>0</v>
       </c>
       <c r="L63" s="5"/>
-      <c r="M63" s="26"/>
+      <c r="M63" s="24"/>
       <c r="N63" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="O63">
         <v>8</v>
@@ -3605,9 +3605,9 @@
       </c>
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A64" s="26"/>
+      <c r="A64" s="24"/>
       <c r="B64" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C64">
         <v>1500</v>
@@ -3620,9 +3620,9 @@
         <v>0</v>
       </c>
       <c r="F64" s="5"/>
-      <c r="G64" s="26"/>
+      <c r="G64" s="24"/>
       <c r="H64" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I64">
         <v>1500</v>
@@ -3635,10 +3635,10 @@
         <v>0</v>
       </c>
       <c r="L64" s="5"/>
-      <c r="N64" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="O64" s="24"/>
+      <c r="N64" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="O64" s="27"/>
       <c r="P64" s="5"/>
       <c r="Q64" s="21">
         <f>SUM(Q51:Q63)</f>
@@ -3646,9 +3646,9 @@
       </c>
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A65" s="26"/>
+      <c r="A65" s="24"/>
       <c r="B65" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C65">
         <v>4000</v>
@@ -3661,9 +3661,9 @@
         <v>0</v>
       </c>
       <c r="F65" s="5"/>
-      <c r="G65" s="26"/>
+      <c r="G65" s="24"/>
       <c r="H65" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I65">
         <v>4000</v>
@@ -3676,17 +3676,17 @@
         <v>0</v>
       </c>
       <c r="L65" s="5"/>
-      <c r="N65" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="O65" s="26"/>
-      <c r="P65" s="26"/>
+      <c r="N65" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="O65" s="24"/>
+      <c r="P65" s="24"/>
       <c r="Q65" s="16"/>
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A66" s="26"/>
+      <c r="A66" s="24"/>
       <c r="B66" s="9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C66">
         <v>4000</v>
@@ -3699,9 +3699,9 @@
         <v>0</v>
       </c>
       <c r="F66" s="5"/>
-      <c r="G66" s="26"/>
+      <c r="G66" s="24"/>
       <c r="H66" s="9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I66">
         <v>4000</v>
@@ -3714,18 +3714,18 @@
         <v>0</v>
       </c>
       <c r="L66" s="5"/>
-      <c r="N66" s="24"/>
-      <c r="O66" s="24"/>
-      <c r="P66" s="24"/>
+      <c r="N66" s="27"/>
+      <c r="O66" s="27"/>
+      <c r="P66" s="27"/>
       <c r="Q66" s="11">
         <f>SUM(Q64+Q50+Q27)</f>
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A67" s="26"/>
+      <c r="A67" s="24"/>
       <c r="B67" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C67">
         <v>25000</v>
@@ -3738,9 +3738,9 @@
         <v>0</v>
       </c>
       <c r="F67" s="5"/>
-      <c r="G67" s="26"/>
+      <c r="G67" s="24"/>
       <c r="H67" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I67">
         <v>25000</v>
@@ -3755,9 +3755,9 @@
       <c r="L67" s="5"/>
     </row>
     <row r="68" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A68" s="26"/>
+      <c r="A68" s="24"/>
       <c r="B68" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C68">
         <v>1</v>
@@ -3770,9 +3770,9 @@
         <v>0</v>
       </c>
       <c r="F68" s="5"/>
-      <c r="G68" s="26"/>
+      <c r="G68" s="24"/>
       <c r="H68" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I68">
         <v>1</v>
@@ -3787,9 +3787,9 @@
       <c r="L68" s="5"/>
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A69" s="26"/>
+      <c r="A69" s="24"/>
       <c r="B69" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C69">
         <v>50000</v>
@@ -3802,9 +3802,9 @@
         <v>0</v>
       </c>
       <c r="F69" s="5"/>
-      <c r="G69" s="26"/>
+      <c r="G69" s="24"/>
       <c r="H69" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I69">
         <v>50000</v>
@@ -3819,9 +3819,9 @@
       <c r="L69" s="5"/>
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A70" s="26"/>
+      <c r="A70" s="24"/>
       <c r="B70" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -3834,9 +3834,9 @@
         <v>0</v>
       </c>
       <c r="F70" s="5"/>
-      <c r="G70" s="26"/>
+      <c r="G70" s="24"/>
       <c r="H70" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I70">
         <v>1</v>
@@ -3851,9 +3851,9 @@
       <c r="L70" s="5"/>
     </row>
     <row r="71" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="26"/>
+      <c r="A71" s="24"/>
       <c r="B71" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C71">
         <v>10000</v>
@@ -3866,9 +3866,9 @@
         <v>0</v>
       </c>
       <c r="F71" s="5"/>
-      <c r="G71" s="26"/>
+      <c r="G71" s="24"/>
       <c r="H71" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I71">
         <v>10000</v>
@@ -3883,9 +3883,9 @@
       <c r="L71" s="5"/>
     </row>
     <row r="72" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A72" s="26"/>
+      <c r="A72" s="24"/>
       <c r="B72" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C72">
         <v>40000</v>
@@ -3898,9 +3898,9 @@
         <v>0</v>
       </c>
       <c r="F72" s="5"/>
-      <c r="G72" s="26"/>
+      <c r="G72" s="24"/>
       <c r="H72" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I72">
         <v>40000</v>
@@ -3915,20 +3915,20 @@
       <c r="L72" s="5"/>
     </row>
     <row r="73" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B73" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="C73" s="24"/>
+      <c r="B73" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C73" s="27"/>
       <c r="D73" s="5"/>
       <c r="E73" s="21">
         <f>SUM(E62:E72)</f>
         <v>0</v>
       </c>
       <c r="F73" s="22"/>
-      <c r="H73" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="I73" s="24"/>
+      <c r="H73" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="I73" s="27"/>
       <c r="J73" s="5"/>
       <c r="K73" s="21">
         <f>SUM(K62:K72)</f>
@@ -3938,10 +3938,10 @@
     </row>
     <row r="74" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A74" s="25" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C74">
         <v>12</v>
@@ -3955,10 +3955,10 @@
       </c>
       <c r="F74" s="5"/>
       <c r="G74" s="25" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I74">
         <v>12</v>
@@ -3973,9 +3973,9 @@
       <c r="L74" s="5"/>
     </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A75" s="26"/>
+      <c r="A75" s="24"/>
       <c r="B75" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C75">
         <v>12</v>
@@ -3988,9 +3988,9 @@
         <v>0</v>
       </c>
       <c r="F75" s="5"/>
-      <c r="G75" s="26"/>
+      <c r="G75" s="24"/>
       <c r="H75" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I75">
         <v>12</v>
@@ -4005,9 +4005,9 @@
       <c r="L75" s="5"/>
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A76" s="26"/>
+      <c r="A76" s="24"/>
       <c r="B76" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C76">
         <v>37500</v>
@@ -4020,9 +4020,9 @@
         <v>0</v>
       </c>
       <c r="F76" s="5"/>
-      <c r="G76" s="26"/>
+      <c r="G76" s="24"/>
       <c r="H76" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I76">
         <v>37500</v>
@@ -4037,9 +4037,9 @@
       <c r="L76" s="5"/>
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A77" s="26"/>
+      <c r="A77" s="24"/>
       <c r="B77" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C77">
         <v>1</v>
@@ -4052,9 +4052,9 @@
         <v>0</v>
       </c>
       <c r="F77" s="5"/>
-      <c r="G77" s="26"/>
+      <c r="G77" s="24"/>
       <c r="H77" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I77">
         <v>1</v>
@@ -4069,9 +4069,9 @@
       <c r="L77" s="5"/>
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A78" s="26"/>
+      <c r="A78" s="24"/>
       <c r="B78" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C78">
         <v>50000</v>
@@ -4084,9 +4084,9 @@
         <v>0</v>
       </c>
       <c r="F78" s="5"/>
-      <c r="G78" s="26"/>
+      <c r="G78" s="24"/>
       <c r="H78" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I78">
         <v>50000</v>
@@ -4101,9 +4101,9 @@
       <c r="L78" s="5"/>
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A79" s="26"/>
+      <c r="A79" s="24"/>
       <c r="B79" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C79">
         <v>1</v>
@@ -4116,9 +4116,9 @@
         <v>0</v>
       </c>
       <c r="F79" s="5"/>
-      <c r="G79" s="26"/>
+      <c r="G79" s="24"/>
       <c r="H79" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I79">
         <v>1</v>
@@ -4133,9 +4133,9 @@
       <c r="L79" s="5"/>
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A80" s="26"/>
+      <c r="A80" s="24"/>
       <c r="B80" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C80">
         <v>10000</v>
@@ -4148,9 +4148,9 @@
         <v>0</v>
       </c>
       <c r="F80" s="5"/>
-      <c r="G80" s="26"/>
+      <c r="G80" s="24"/>
       <c r="H80" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I80">
         <v>10000</v>
@@ -4165,9 +4165,9 @@
       <c r="L80" s="5"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A81" s="26"/>
+      <c r="A81" s="24"/>
       <c r="B81" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C81">
         <v>40000</v>
@@ -4180,9 +4180,9 @@
         <v>0</v>
       </c>
       <c r="F81" s="5"/>
-      <c r="G81" s="26"/>
+      <c r="G81" s="24"/>
       <c r="H81" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I81">
         <v>40000</v>
@@ -4197,9 +4197,9 @@
       <c r="L81" s="5"/>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A82" s="26"/>
+      <c r="A82" s="24"/>
       <c r="B82" s="9" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C82">
         <v>8</v>
@@ -4212,9 +4212,9 @@
         <v>0</v>
       </c>
       <c r="F82" s="5"/>
-      <c r="G82" s="26"/>
+      <c r="G82" s="24"/>
       <c r="H82" s="9" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I82">
         <v>8</v>
@@ -4229,9 +4229,9 @@
       <c r="L82" s="5"/>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A83" s="26"/>
+      <c r="A83" s="24"/>
       <c r="B83" s="9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C83">
         <v>500</v>
@@ -4244,9 +4244,9 @@
         <v>0</v>
       </c>
       <c r="F83" s="5"/>
-      <c r="G83" s="26"/>
+      <c r="G83" s="24"/>
       <c r="H83" s="9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I83">
         <v>500</v>
@@ -4261,9 +4261,9 @@
       <c r="L83" s="5"/>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A84" s="26"/>
+      <c r="A84" s="24"/>
       <c r="B84" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C84">
         <v>60000</v>
@@ -4276,9 +4276,9 @@
         <v>0</v>
       </c>
       <c r="F84" s="5"/>
-      <c r="G84" s="26"/>
+      <c r="G84" s="24"/>
       <c r="H84" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I84">
         <v>60000</v>
@@ -4293,20 +4293,20 @@
       <c r="L84" s="5"/>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B85" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="C85" s="24"/>
+      <c r="B85" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C85" s="27"/>
       <c r="D85" s="5"/>
       <c r="E85" s="16">
         <f>SUM(E74:E84)</f>
         <v>0</v>
       </c>
       <c r="F85" s="5"/>
-      <c r="H85" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="I85" s="24"/>
+      <c r="H85" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="I85" s="27"/>
       <c r="J85" s="5"/>
       <c r="K85" s="16">
         <f>SUM(K74:K84)</f>
@@ -4315,33 +4315,33 @@
       <c r="L85" s="5"/>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B86" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="C86" s="26"/>
-      <c r="D86" s="26"/>
+      <c r="B86" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="C86" s="24"/>
+      <c r="D86" s="24"/>
       <c r="E86" s="16"/>
       <c r="F86" s="5"/>
-      <c r="H86" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="I86" s="26"/>
-      <c r="J86" s="26"/>
+      <c r="H86" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="I86" s="24"/>
+      <c r="J86" s="24"/>
       <c r="K86" s="16"/>
       <c r="L86" s="5"/>
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B87" s="24"/>
-      <c r="C87" s="24"/>
-      <c r="D87" s="24"/>
+      <c r="B87" s="27"/>
+      <c r="C87" s="27"/>
+      <c r="D87" s="27"/>
       <c r="E87" s="11">
         <f>SUM(E85+E73+E61+E46+E32+E19)</f>
         <v>0</v>
       </c>
       <c r="F87" s="10"/>
-      <c r="H87" s="24"/>
-      <c r="I87" s="24"/>
-      <c r="J87" s="24"/>
+      <c r="H87" s="27"/>
+      <c r="I87" s="27"/>
+      <c r="J87" s="27"/>
       <c r="K87" s="11">
         <f>SUM(K85+K73+K61+K46+K32+K19)</f>
         <v>0</v>
@@ -4350,15 +4350,20 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:K1"/>
-    <mergeCell ref="M28:M48"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="G20:G31"/>
-    <mergeCell ref="H85:I85"/>
-    <mergeCell ref="G33:G45"/>
-    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="N65:P66"/>
+    <mergeCell ref="A74:A84"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="A6:A18"/>
+    <mergeCell ref="G62:G72"/>
+    <mergeCell ref="A33:A45"/>
+    <mergeCell ref="A62:A72"/>
+    <mergeCell ref="A20:A31"/>
+    <mergeCell ref="A47:A59"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="M6:M26"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="M51:M63"/>
+    <mergeCell ref="N27:O27"/>
     <mergeCell ref="B86:D87"/>
     <mergeCell ref="B73:C73"/>
     <mergeCell ref="G47:G59"/>
@@ -4375,21 +4380,16 @@
     <mergeCell ref="H32:I32"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="M4:O4"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="G1:K1"/>
+    <mergeCell ref="M28:M48"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="G20:G31"/>
+    <mergeCell ref="H85:I85"/>
+    <mergeCell ref="G33:G45"/>
+    <mergeCell ref="H61:I61"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="A47:A59"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="M6:M26"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="M51:M63"/>
-    <mergeCell ref="A74:A84"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="A6:A18"/>
-    <mergeCell ref="G62:G72"/>
-    <mergeCell ref="A33:A45"/>
-    <mergeCell ref="A62:A72"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="A20:A31"/>
-    <mergeCell ref="N65:P66"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B1" location="Sheet1!B4" tooltip="Jump to TOP CEO EVENT" display="TOP CEO EVENT" xr:uid="{00000000-0004-0000-0000-000000000000}"/>

</xml_diff>